<commit_message>
Remove remaining long dashes in migration and UAT spreadsheets
</commit_message>
<xml_diff>
--- a/assets/files/Data_Migration_Workbook.xlsx
+++ b/assets/files/Data_Migration_Workbook.xlsx
@@ -2,20 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Overview" sheetId="1" r:id="R257d399beeb942d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Data_Inventory" sheetId="2" r:id="Rf897f0332b1843e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Source_Target_Map" sheetId="3" r:id="R71be7813e54242b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Profile_Summary" sheetId="4" r:id="Re02bfc2ea73e4796"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Cleansing_Log" sheetId="5" r:id="R6f782dd6c1424804"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Migration_Validation" sheetId="6" r:id="R6cd34caad3814d48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Reconciliation" sheetId="7" r:id="Rd0cbc99507804a77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Exception_Detail" sheetId="8" r:id="R08c66890ab49432f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Data_Controls" sheetId="9" r:id="Rcad397eec3364c5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Customer_Sample" sheetId="10" r:id="R8fc63b16d5ee4cb3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Inventory_Sample" sheetId="11" r:id="Rec2750b3fb6e4338"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Generation_Record" sheetId="12" r:id="R172a776254dd4df7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Readiness_Gate" sheetId="13" r:id="R4ea5140463574f94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99_Lists" sheetId="14" r:id="R2789e0c50fb34b54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Overview" sheetId="1" r:id="Rb79c01d41dbf4312"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Data_Inventory" sheetId="2" r:id="R23ed9467557d46c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Source_Target_Map" sheetId="3" r:id="Refcc94ff16f1487b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Profile_Summary" sheetId="4" r:id="Rcc4cd1f37b1c49e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Cleansing_Log" sheetId="5" r:id="R5b4af0c985dd4bec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Migration_Validation" sheetId="6" r:id="R66d14f6442e74d4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07_Reconciliation" sheetId="7" r:id="R336239ca16f147af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_Exception_Detail" sheetId="8" r:id="R3f0915c213f5451a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_Data_Controls" sheetId="9" r:id="Rcea28e2e9101462f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_Customer_Sample" sheetId="10" r:id="R75af7c1fc9a84c2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_Inventory_Sample" sheetId="11" r:id="R422539ae7ef0401d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_Generation_Record" sheetId="12" r:id="R6ad9d76664b24297"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_Readiness_Gate" sheetId="13" r:id="R0a2353bc55524a44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99_Lists" sheetId="14" r:id="Rbed4e72114564c56"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -305,9 +305,7 @@
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="48672768"/>
-        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
         <c:axId val="48672768"/>
@@ -372,7 +370,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5fd70636fc54431b"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rff9ba77a4951485b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -867,7 +865,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc457a5f285cd4c62"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf51ea1abf6d047a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1301,7 +1299,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26c0e053b6bf4675"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22855758eea84618"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1808,7 +1806,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Red0182afed704e45"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2701c52b7aca4388"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2036,7 +2034,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c8ecb12545d48b3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c6ea85f2a074f7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2183,7 +2181,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra663cf83fecd4fab"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1f59484cae624feb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2627,7 +2625,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2baa97eb91f843cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2eba5f2ed92341d7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3778,7 +3776,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0b1dac2dc284693"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf4c1746adff74168"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4099,9 +4097,9 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe79a03172244204"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc465ce07845644af"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R003be1f8a5824ddd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdf86586fab504d76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4364,7 +4362,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6af018c35d724486"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbaf5031cfc434f7c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4795,7 +4793,7 @@
         <x:v>Customer/plan/work-order critical rejections remain</x:v>
       </x:c>
       <x:c r="F20" s="33" t="str">
-        <x:v>FAIL — remediation required</x:v>
+        <x:v>FAIL - remediation required</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
@@ -4826,7 +4824,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3fec6fe2656466c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28ed263403bd4c86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5094,7 +5092,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3fbbc18d8afa420b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b8b00781c4a4a10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6406,7 +6404,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R301ffeb8a87b412c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19db1c85503d497e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6660,7 +6658,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7011872d1b824267"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f67f2a4cd744a17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>